<commit_message>
+  redmine Bug #5947
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/WEB-INF/templates/sc/loa/specification.xlsx
+++ b/portlets/NGeP-portlet/docroot/WEB-INF/templates/sc/loa/specification.xlsx
@@ -4,18 +4,19 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4506"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13545" windowHeight="4500"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="14670" windowHeight="3180" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ProductSheet" sheetId="1" r:id="rId1"/>
     <sheet name="ServiceSheet" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="125725"/>
+  <oleSize ref="A1:K9"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
   <si>
     <t>Item</t>
   </si>
@@ -39,12 +40,6 @@
   </si>
   <si>
     <t>Specification</t>
-  </si>
-  <si>
-    <t>Answer Remarks</t>
-  </si>
-  <si>
-    <t>Answer Text</t>
   </si>
 </sst>
 </file>
@@ -420,12 +415,8 @@
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -472,12 +463,8 @@
       <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
   </sheetData>

</xml_diff>